<commit_message>
swapping with original master deck, naming convention, case study crated using ai adding to existing excel, editing downloaded file
</commit_message>
<xml_diff>
--- a/data/registry/J2W_CaseStudy_Portfolio_Metadata.xlsx
+++ b/data/registry/J2W_CaseStudy_Portfolio_Metadata.xlsx
@@ -749,7 +749,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:K137"/>
+  <dimension ref="A1:Q151"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="9" customWidth="1" style="17" min="1" max="1"/>
@@ -820,6 +820,36 @@
           <t>title</t>
         </is>
       </c>
+      <c r="L1" s="17" t="inlineStr">
+        <is>
+          <t>include_rule_legacy</t>
+        </is>
+      </c>
+      <c r="M1" s="17" t="inlineStr">
+        <is>
+          <t>stage_intro</t>
+        </is>
+      </c>
+      <c r="N1" s="17" t="inlineStr">
+        <is>
+          <t>stage_first</t>
+        </is>
+      </c>
+      <c r="O1" s="17" t="inlineStr">
+        <is>
+          <t>stage_second</t>
+        </is>
+      </c>
+      <c r="P1" s="17" t="inlineStr">
+        <is>
+          <t>composition</t>
+        </is>
+      </c>
+      <c r="Q1" s="17" t="inlineStr">
+        <is>
+          <t>trigger</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="30" customHeight="1" s="18">
       <c r="A2" s="24" t="inlineStr">
@@ -861,6 +891,11 @@
           <t>BUSINESS DRIVERS| TECHNOLOGY ACCELERATORS | GAME CHANGERS</t>
         </is>
       </c>
+      <c r="L2" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="30" customHeight="1" s="18">
       <c r="A3" s="24" t="inlineStr">
@@ -885,7 +920,7 @@
       </c>
       <c r="E3" s="27" t="inlineStr">
         <is>
-          <t>ALWAYS</t>
+          <t>SPECIAL - see matcher._SPECIAL_STAGE_RULES</t>
         </is>
       </c>
       <c r="F3" s="25" t="n"/>
@@ -902,6 +937,21 @@
           <t>WHO WE ARE</t>
         </is>
       </c>
+      <c r="L3" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+      <c r="N3" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O3" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="30" customHeight="1" s="18">
       <c r="A4" s="24" t="inlineStr">
@@ -926,7 +976,7 @@
       </c>
       <c r="E4" s="27" t="inlineStr">
         <is>
-          <t>ALWAYS</t>
+          <t>STAGE_RULE (stage=-YY, wt=None, trigger=none)</t>
         </is>
       </c>
       <c r="F4" s="25" t="n"/>
@@ -943,6 +993,21 @@
           <t>Architects of Transformation</t>
         </is>
       </c>
+      <c r="L4" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+      <c r="N4" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O4" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="30" customHeight="1" s="18">
       <c r="A5" s="24" t="inlineStr">
@@ -967,7 +1032,7 @@
       </c>
       <c r="E5" s="27" t="inlineStr">
         <is>
-          <t>ALWAYS</t>
+          <t>SPECIAL - see matcher._SPECIAL_STAGE_RULES</t>
         </is>
       </c>
       <c r="F5" s="25" t="n"/>
@@ -988,6 +1053,11 @@
           <t>WHAT WE OFFER</t>
         </is>
       </c>
+      <c r="L5" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="30" customHeight="1" s="18">
       <c r="A6" s="24" t="inlineStr">
@@ -1012,7 +1082,7 @@
       </c>
       <c r="E6" s="27" t="inlineStr">
         <is>
-          <t>ALWAYS</t>
+          <t>STAGE_RULE (stage=-YY, wt=None, trigger=none)</t>
         </is>
       </c>
       <c r="F6" s="25" t="n"/>
@@ -1029,6 +1099,21 @@
           <t>THE J2W OPERATING MODEL</t>
         </is>
       </c>
+      <c r="L6" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+      <c r="N6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O6" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="30" customHeight="1" s="18">
       <c r="A7" s="24" t="inlineStr">
@@ -1070,6 +1155,11 @@
           <t>WHAT WE OWN</t>
         </is>
       </c>
+      <c r="L7" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="30" customHeight="1" s="18">
       <c r="A8" s="24" t="inlineStr">
@@ -1094,10 +1184,14 @@
       </c>
       <c r="E8" s="27" t="inlineStr">
         <is>
-          <t>ALWAYS</t>
-        </is>
-      </c>
-      <c r="F8" s="25" t="n"/>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE,AI_POD, trigger=none)</t>
+        </is>
+      </c>
+      <c r="F8" s="25" t="inlineStr">
+        <is>
+          <t>WORKFORCE,AI_POD</t>
+        </is>
+      </c>
       <c r="G8" s="25" t="n"/>
       <c r="H8" s="25" t="n"/>
       <c r="I8" s="27" t="n"/>
@@ -1109,6 +1203,21 @@
       <c r="K8" s="27" t="inlineStr">
         <is>
           <t>NEXT STEPS</t>
+        </is>
+      </c>
+      <c r="L8" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+      <c r="N8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O8" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
         </is>
       </c>
     </row>
@@ -1152,6 +1261,11 @@
           <t>"Let's win together"</t>
         </is>
       </c>
+      <c r="L9" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="30" customHeight="1" s="18">
       <c r="A10" s="24" t="inlineStr">
@@ -1197,6 +1311,11 @@
           <t>01</t>
         </is>
       </c>
+      <c r="L10" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes WORKFORCE</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="30" customHeight="1" s="18">
       <c r="A11" s="24" t="inlineStr">
@@ -1221,7 +1340,7 @@
       </c>
       <c r="E11" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes WORKFORCE</t>
+          <t>STAGE_RULE (stage=YYY, wt=WORKFORCE, trigger=none)</t>
         </is>
       </c>
       <c r="F11" s="25" t="inlineStr">
@@ -1242,6 +1361,26 @@
           <t>Sourcing Engine</t>
         </is>
       </c>
+      <c r="L11" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes WORKFORCE</t>
+        </is>
+      </c>
+      <c r="M11" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N11" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O11" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="30" customHeight="1" s="18">
       <c r="A12" s="24" t="inlineStr">
@@ -1266,7 +1405,7 @@
       </c>
       <c r="E12" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes WORKFORCE</t>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
         </is>
       </c>
       <c r="F12" s="25" t="inlineStr">
@@ -1287,6 +1426,16 @@
           <t>WORKFORCE SOLUTIONS - HOW WE DELIVER</t>
         </is>
       </c>
+      <c r="L12" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes WORKFORCE</t>
+        </is>
+      </c>
+      <c r="Q12" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="30" customHeight="1" s="18">
       <c r="A13" s="24" t="inlineStr">
@@ -1311,7 +1460,7 @@
       </c>
       <c r="E13" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes WORKFORCE</t>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
         </is>
       </c>
       <c r="F13" s="25" t="inlineStr">
@@ -1332,6 +1481,26 @@
           <t>STRUCTURAL DIFFERENTIATION</t>
         </is>
       </c>
+      <c r="L13" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes WORKFORCE</t>
+        </is>
+      </c>
+      <c r="N13" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O13" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q13" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="30" customHeight="1" s="18">
       <c r="A14" s="24" t="inlineStr">
@@ -1356,7 +1525,7 @@
       </c>
       <c r="E14" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes WORKFORCE</t>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
         </is>
       </c>
       <c r="F14" s="25" t="inlineStr">
@@ -1379,6 +1548,26 @@
       <c r="K14" s="27" t="inlineStr">
         <is>
           <t>WHY J2W - NOT THE BIG 4 OR LARGE SIs</t>
+        </is>
+      </c>
+      <c r="L14" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes WORKFORCE</t>
+        </is>
+      </c>
+      <c r="N14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O14" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q14" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
         </is>
       </c>
     </row>
@@ -1426,6 +1615,11 @@
           <t>02</t>
         </is>
       </c>
+      <c r="L15" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes AI_POD</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="30" customHeight="1" s="18">
       <c r="A16" s="24" t="inlineStr">
@@ -1450,7 +1644,7 @@
       </c>
       <c r="E16" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes AI_POD</t>
+          <t>SPECIAL - see matcher._SPECIAL_STAGE_RULES</t>
         </is>
       </c>
       <c r="F16" s="25" t="inlineStr">
@@ -1471,6 +1665,11 @@
           <t>Introducing the AI-First Pod Model</t>
         </is>
       </c>
+      <c r="L16" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes AI_POD</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="30" customHeight="1" s="18">
       <c r="A17" s="24" t="inlineStr">
@@ -1495,7 +1694,7 @@
       </c>
       <c r="E17" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes AI_POD</t>
+          <t>SPECIAL - see matcher._SPECIAL_STAGE_RULES</t>
         </is>
       </c>
       <c r="F17" s="25" t="inlineStr">
@@ -1516,6 +1715,11 @@
           <t>The J2W AI Research Wing</t>
         </is>
       </c>
+      <c r="L17" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes AI_POD</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="30" customHeight="1" s="18">
       <c r="A18" s="24" t="inlineStr">
@@ -1561,6 +1765,11 @@
           <t>03</t>
         </is>
       </c>
+      <c r="L18" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes MS</t>
+        </is>
+      </c>
     </row>
     <row r="19" ht="30" customHeight="1" s="18">
       <c r="A19" s="24" t="inlineStr">
@@ -1585,7 +1794,7 @@
       </c>
       <c r="E19" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes MS</t>
+          <t>STAGE_RULE (stage=-YY, wt=MS, trigger=none)</t>
         </is>
       </c>
       <c r="F19" s="25" t="inlineStr">
@@ -1606,6 +1815,21 @@
           <t>Managed Service Solutions</t>
         </is>
       </c>
+      <c r="L19" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes MS</t>
+        </is>
+      </c>
+      <c r="N19" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O19" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="20" ht="30" customHeight="1" s="18">
       <c r="A20" s="24" t="inlineStr">
@@ -1630,7 +1854,7 @@
       </c>
       <c r="E20" s="27" t="inlineStr">
         <is>
-          <t>IF work_type includes MS</t>
+          <t>STAGE_RULE (stage=-YY, wt=MS, trigger=none)</t>
         </is>
       </c>
       <c r="F20" s="25" t="inlineStr">
@@ -1651,6 +1875,21 @@
           <t>Strategic Managed Services Offerings</t>
         </is>
       </c>
+      <c r="L20" s="17" t="inlineStr">
+        <is>
+          <t>IF work_type includes MS</t>
+        </is>
+      </c>
+      <c r="N20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O20" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
     </row>
     <row r="21" ht="30" customHeight="1" s="18">
       <c r="A21" s="24" t="inlineStr">
@@ -1696,6 +1935,11 @@
           <t>J2W</t>
         </is>
       </c>
+      <c r="L21" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
     </row>
     <row r="22" ht="30" customHeight="1" s="18">
       <c r="A22" s="24" t="inlineStr">
@@ -1737,6 +1981,11 @@
           <t>AI PODS • J2W DELIVERY</t>
         </is>
       </c>
+      <c r="L22" s="17" t="inlineStr">
+        <is>
+          <t>IF &gt;=1 AI_POD case selected</t>
+        </is>
+      </c>
     </row>
     <row r="23" ht="30" customHeight="1" s="18">
       <c r="A23" s="24" t="inlineStr">
@@ -1790,6 +2039,11 @@
           <t>AI-FIRST POD DELIVERY — GE HEALTHCARE ENGINEERING</t>
         </is>
       </c>
+      <c r="L23" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="24" ht="30" customHeight="1" s="18">
       <c r="A24" s="24" t="inlineStr">
@@ -1843,6 +2097,11 @@
           <t>CAAS GLOBAL MEDTECH ENGINEERING</t>
         </is>
       </c>
+      <c r="L24" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="30" customHeight="1" s="18">
       <c r="A25" s="24" t="inlineStr">
@@ -1896,6 +2155,11 @@
           <t>GCC ENABLEMENT — HANDHELD ULTRASOUND (MEDTECH)</t>
         </is>
       </c>
+      <c r="L25" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="26" ht="30" customHeight="1" s="18">
       <c r="A26" s="24" t="inlineStr">
@@ -1949,6 +2213,11 @@
           <t>MAMMOGRAPHY EXCELLENCE — AI-ENHANCED DIAGNOSTICS</t>
         </is>
       </c>
+      <c r="L26" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="30" customHeight="1" s="18">
       <c r="A27" s="24" t="inlineStr">
@@ -2002,6 +2271,11 @@
           <t>PATIENT CARE SOLUTIONS — MOBILE APP &amp; DEVSECOPS</t>
         </is>
       </c>
+      <c r="L27" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="28" ht="30" customHeight="1" s="18">
       <c r="A28" s="24" t="inlineStr">
@@ -2055,6 +2329,11 @@
           <t>CAAS GLOBAL AUTOMOTIVE OEM ENGINEERING</t>
         </is>
       </c>
+      <c r="L28" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="29" ht="30" customHeight="1" s="18">
       <c r="A29" s="24" t="inlineStr">
@@ -2108,6 +2387,11 @@
           <t>CYBERSECURITY — PENTESTING TO COMPLIANCE</t>
         </is>
       </c>
+      <c r="L29" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="30" customHeight="1" s="18">
       <c r="A30" s="24" t="inlineStr">
@@ -2161,6 +2445,11 @@
           <t>APP STORE RATING RECOVERY FOR DIGITAL BANK</t>
         </is>
       </c>
+      <c r="L30" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="31" ht="30" customHeight="1" s="18">
       <c r="A31" s="24" t="inlineStr">
@@ -2214,6 +2503,11 @@
           <t>DEVSECOPS PIPELINE FOR OPEN BANKING</t>
         </is>
       </c>
+      <c r="L31" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="32" ht="30" customHeight="1" s="18">
       <c r="A32" s="24" t="inlineStr">
@@ -2267,6 +2561,11 @@
           <t>MANAGED TESTING FOR OTT PLATFORM LAUNCH — US TELECOM</t>
         </is>
       </c>
+      <c r="L32" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="33" ht="30" customHeight="1" s="18">
       <c r="A33" s="24" t="inlineStr">
@@ -2320,6 +2619,11 @@
           <t>SAP PERFORMANCE TESTING FOR HIGH-LOAD HEALTH INSURANCE</t>
         </is>
       </c>
+      <c r="L33" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="34" ht="30" customHeight="1" s="18">
       <c r="A34" s="24" t="inlineStr">
@@ -2373,6 +2677,11 @@
           <t>E-LEARNING AUTOMATION FOR LEADING EDTECH PROVIDER</t>
         </is>
       </c>
+      <c r="L34" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="30" customHeight="1" s="18">
       <c r="A35" s="24" t="inlineStr">
@@ -2424,6 +2733,11 @@
       <c r="K35" s="27" t="inlineStr">
         <is>
           <t>NEXT-GENERATION GAMING CONSOLE ENGINEERING</t>
+        </is>
+      </c>
+      <c r="L35" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
         </is>
       </c>
     </row>
@@ -2467,6 +2781,11 @@
           <t>WORKFORCE SOLUTIONS • J2W DELIVERY</t>
         </is>
       </c>
+      <c r="L36" s="17" t="inlineStr">
+        <is>
+          <t>IF &gt;=1 WORKFORCE case selected</t>
+        </is>
+      </c>
     </row>
     <row r="37" ht="30" customHeight="1" s="18">
       <c r="A37" s="24" t="inlineStr">
@@ -2520,6 +2839,11 @@
           <t>RAPID SECURE ODC DEPLOYMENT</t>
         </is>
       </c>
+      <c r="L37" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="30" customHeight="1" s="18">
       <c r="A38" s="24" t="inlineStr">
@@ -2573,6 +2897,11 @@
           <t>GREENFIELD AI-READY GCC BUILD — MAJOR US AIRLINE</t>
         </is>
       </c>
+      <c r="L38" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="39" ht="30" customHeight="1" s="18">
       <c r="A39" s="24" t="inlineStr">
@@ -2626,6 +2955,11 @@
           <t>GREENFIELD TO APAC INNOVATION HUB — 15-YEAR BFSI EVOLUTION</t>
         </is>
       </c>
+      <c r="L39" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="40" ht="30" customHeight="1" s="18">
       <c r="A40" s="24" t="inlineStr">
@@ -2679,6 +3013,11 @@
           <t>FINANCE &amp; TECHNOLOGY COE BUILD — GLOBAL INDUSTRIAL LEADER (SULZER)</t>
         </is>
       </c>
+      <c r="L40" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="41" ht="30" customHeight="1" s="18">
       <c r="A41" s="24" t="inlineStr">
@@ -2732,6 +3071,11 @@
           <t>ZERO-DISRUPTION WORKFORCE SCALING FOR HEALTHCARE IT</t>
         </is>
       </c>
+      <c r="L41" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="42" ht="30" customHeight="1" s="18">
       <c r="A42" s="24" t="inlineStr">
@@ -2785,6 +3129,11 @@
           <t>CA &amp; FINANCE TALENT PIPELINE — GLOBAL ALTERNATIVE ASSET MANAGER</t>
         </is>
       </c>
+      <c r="L42" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="43" ht="30" customHeight="1" s="18">
       <c r="A43" s="24" t="inlineStr">
@@ -2834,6 +3183,11 @@
           <t>CORE BANKING TRANSFORMATION &amp; SUPPORT OPTIMIZATION</t>
         </is>
       </c>
+      <c r="L43" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="44" ht="30" customHeight="1" s="18">
       <c r="A44" s="24" t="inlineStr">
@@ -2887,6 +3241,11 @@
           <t>CLOUD MIGRATION &amp; 24x7 INFRASTRUCTURE SUPPORT</t>
         </is>
       </c>
+      <c r="L44" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="30" customHeight="1" s="18">
       <c r="A45" s="24" t="inlineStr">
@@ -2934,6 +3293,11 @@
       <c r="K45" s="27" t="inlineStr">
         <is>
           <t>GLOBAL PHARMACEUTICAL PROCESS EXCELLENCE</t>
+        </is>
+      </c>
+      <c r="L45" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
         </is>
       </c>
     </row>
@@ -2977,6 +3341,11 @@
           <t>AI CASE STUDY PORTFOLIO • J2W DELIVERY</t>
         </is>
       </c>
+      <c r="L46" s="17" t="inlineStr">
+        <is>
+          <t>IF &gt;=1 portfolio case selected</t>
+        </is>
+      </c>
     </row>
     <row r="47" ht="30" customHeight="1" s="18">
       <c r="A47" s="24" t="inlineStr">
@@ -3030,6 +3399,11 @@
           <t>PROCUREMENT CYCLE COMPRESSION</t>
         </is>
       </c>
+      <c r="L47" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="48" ht="30" customHeight="1" s="18">
       <c r="A48" s="24" t="inlineStr">
@@ -3083,6 +3457,11 @@
           <t>DEMAND-DRIVEN MATERIAL PLANNING</t>
         </is>
       </c>
+      <c r="L48" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="49" ht="30" customHeight="1" s="18">
       <c r="A49" s="24" t="inlineStr">
@@ -3136,6 +3515,11 @@
           <t>NX CAD TOOLKIT &amp; MACRO CONSOLIDATION</t>
         </is>
       </c>
+      <c r="L49" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="50" ht="30" customHeight="1" s="18">
       <c r="A50" s="24" t="inlineStr">
@@ -3189,6 +3573,11 @@
           <t>AGENTIC QUALITY ROOT CAUSE INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L50" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="51" ht="30" customHeight="1" s="18">
       <c r="A51" s="24" t="inlineStr">
@@ -3242,6 +3631,11 @@
           <t>SHEET METAL FORMING INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L51" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="52" ht="30" customHeight="1" s="18">
       <c r="A52" s="24" t="inlineStr">
@@ -3295,6 +3689,11 @@
           <t>AERODYNAMIC SIMULATION INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L52" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="53" ht="30" customHeight="1" s="18">
       <c r="A53" s="24" t="inlineStr">
@@ -3348,6 +3747,11 @@
           <t>PREDICTIVE O&amp;M INTELLIGENCE FOR RENEWABLE ASSETS</t>
         </is>
       </c>
+      <c r="L53" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="54" ht="30" customHeight="1" s="18">
       <c r="A54" s="24" t="inlineStr">
@@ -3401,6 +3805,11 @@
           <t>AI ASSISTANT FOR SELL-SIDE EQUITY RESEARCH</t>
         </is>
       </c>
+      <c r="L54" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="30" customHeight="1" s="18">
       <c r="A55" s="24" t="inlineStr">
@@ -3454,6 +3863,11 @@
           <t>MAINFRAME COST OPTIMIZATION — BANKING</t>
         </is>
       </c>
+      <c r="L55" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="30" customHeight="1" s="18">
       <c r="A56" s="24" t="inlineStr">
@@ -3507,6 +3921,11 @@
           <t>DEAL SOURCING INTELLIGENCE — VENTURE CAPITAL</t>
         </is>
       </c>
+      <c r="L56" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="57" ht="30" customHeight="1" s="18">
       <c r="A57" s="24" t="inlineStr">
@@ -3560,6 +3979,11 @@
           <t>AGENTIC INVOICE &amp; CASH MANAGEMENT</t>
         </is>
       </c>
+      <c r="L57" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="58" ht="30" customHeight="1" s="18">
       <c r="A58" s="24" t="inlineStr">
@@ -3613,6 +4037,11 @@
           <t>LOAD BALANCING &amp; DEMAND RESPONSE</t>
         </is>
       </c>
+      <c r="L58" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="59" ht="30" customHeight="1" s="18">
       <c r="A59" s="24" t="inlineStr">
@@ -3666,6 +4095,11 @@
           <t>AIOPS CONTROL TOWER</t>
         </is>
       </c>
+      <c r="L59" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="60" ht="30" customHeight="1" s="18">
       <c r="A60" s="24" t="inlineStr">
@@ -3719,6 +4153,11 @@
           <t>BATTERY ON CLOUD — EV FLEET INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L60" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="61" ht="30" customHeight="1" s="18">
       <c r="A61" s="24" t="inlineStr">
@@ -3770,6 +4209,11 @@
       <c r="K61" s="27" t="inlineStr">
         <is>
           <t>CARBON TRACKING &amp; EMISSION INTELLIGENCE</t>
+        </is>
+      </c>
+      <c r="L61" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
         </is>
       </c>
     </row>
@@ -3809,6 +4253,11 @@
           <t>ARCHITECTS OF TRANSFORMATION</t>
         </is>
       </c>
+      <c r="L62" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — ask user which leaders to show</t>
+        </is>
+      </c>
     </row>
     <row r="63" ht="30" customHeight="1" s="18">
       <c r="A63" s="24" t="inlineStr">
@@ -3850,6 +4299,11 @@
           <t>THE J2W SQUAD</t>
         </is>
       </c>
+      <c r="L63" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — ask user which leaders to show</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="30" customHeight="1" s="18">
       <c r="A64" s="24" t="inlineStr">
@@ -3870,10 +4324,14 @@
       <c r="D64" s="25" t="n"/>
       <c r="E64" s="27" t="inlineStr">
         <is>
-          <t>OPTIONAL — AI decides from transcript, or user asks</t>
-        </is>
-      </c>
-      <c r="F64" s="25" t="n"/>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="F64" s="25" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
       <c r="G64" s="25" t="n"/>
       <c r="H64" s="25" t="n"/>
       <c r="I64" s="27" t="inlineStr">
@@ -3889,6 +4347,26 @@
       <c r="K64" s="27" t="inlineStr">
         <is>
           <t>WORKFORCE SOLUTIONS – WHAT WE DEPLOY</t>
+        </is>
+      </c>
+      <c r="L64" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
+      <c r="N64" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O64" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q64" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
         </is>
       </c>
     </row>
@@ -3928,6 +4406,11 @@
           <t>Workforce Solutions</t>
         </is>
       </c>
+      <c r="L65" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="30" customHeight="1" s="18">
       <c r="A66" s="24" t="inlineStr">
@@ -3948,7 +4431,7 @@
       <c r="D66" s="25" t="n"/>
       <c r="E66" s="27" t="inlineStr">
         <is>
-          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+          <t>MANUAL - filled via client_context module, not registry-driven</t>
         </is>
       </c>
       <c r="F66" s="25" t="n"/>
@@ -3965,6 +4448,11 @@
           <t>Workforce Solutions</t>
         </is>
       </c>
+      <c r="L66" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
     </row>
     <row r="67" ht="30" customHeight="1" s="18">
       <c r="A67" s="24" t="inlineStr">
@@ -3985,7 +4473,7 @@
       <c r="D67" s="25" t="n"/>
       <c r="E67" s="27" t="inlineStr">
         <is>
-          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+          <t>MANUAL - filled via client_context module, not registry-driven</t>
         </is>
       </c>
       <c r="F67" s="25" t="n"/>
@@ -4002,6 +4490,11 @@
           <t>TAILORED APPROACH</t>
         </is>
       </c>
+      <c r="L67" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
     </row>
     <row r="68" ht="30" customHeight="1" s="18">
       <c r="A68" s="24" t="inlineStr">
@@ -4043,6 +4536,11 @@
           <t>WHY J2W - NOT THE BIG 4 OR LARGE SIs</t>
         </is>
       </c>
+      <c r="L68" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="30" customHeight="1" s="18">
       <c r="A69" s="24" t="inlineStr">
@@ -4063,10 +4561,14 @@
       <c r="D69" s="25" t="n"/>
       <c r="E69" s="27" t="inlineStr">
         <is>
-          <t>OPTIONAL — AI decides from transcript, or user asks</t>
-        </is>
-      </c>
-      <c r="F69" s="25" t="n"/>
+          <t>STAGE_RULE (stage=---, wt=AI_POD, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="F69" s="25" t="inlineStr">
+        <is>
+          <t>AI_POD</t>
+        </is>
+      </c>
       <c r="G69" s="25" t="n"/>
       <c r="H69" s="25" t="n"/>
       <c r="I69" s="27" t="n"/>
@@ -4080,6 +4582,16 @@
           <t>AI POD</t>
         </is>
       </c>
+      <c r="L69" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL — AI decides from transcript, or user asks</t>
+        </is>
+      </c>
+      <c r="Q69" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" s="17" t="inlineStr">
@@ -4132,6 +4644,11 @@
           <t>PRE &amp; POST CONTRACT INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L70" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="17" t="inlineStr">
@@ -4184,6 +4701,11 @@
           <t>8D, FMEA AND DOCUMENT INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L71" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="17" t="inlineStr">
@@ -4236,6 +4758,11 @@
           <t>WELD VISION AND JOINT INTEGRITY ANALYTICS</t>
         </is>
       </c>
+      <c r="L72" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="17" t="inlineStr">
@@ -4288,6 +4815,11 @@
           <t>AI-FIRST QUALITY GATES AT INBOUND</t>
         </is>
       </c>
+      <c r="L73" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" s="17" t="inlineStr">
@@ -4340,6 +4872,11 @@
           <t>PREDICTIVE MAINTENANCE INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L74" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="17" t="inlineStr">
@@ -4392,6 +4929,11 @@
           <t>INDUSTRY 4.0 INTELLIGENCE — SPECIALTY CHEMICALS</t>
         </is>
       </c>
+      <c r="L75" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="17" t="inlineStr">
@@ -4444,6 +4986,11 @@
           <t>OPERATIONAL DIGITAL TWIN — OFFSHORE OIL &amp; GAS</t>
         </is>
       </c>
+      <c r="L76" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="17" t="inlineStr">
@@ -4491,6 +5038,11 @@
           <t>ORDER-TO-DELIVERY ENGINE</t>
         </is>
       </c>
+      <c r="L77" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="17" t="inlineStr">
@@ -4543,6 +5095,11 @@
           <t>TOUCHLESS INVOICE PROCESSING</t>
         </is>
       </c>
+      <c r="L78" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="17" t="inlineStr">
@@ -4595,6 +5152,11 @@
           <t>IT-OT CONVERGENCE SECURITY</t>
         </is>
       </c>
+      <c r="L79" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="17" t="inlineStr">
@@ -4647,6 +5209,11 @@
           <t>INTELLIGENT QUALITY ENGINEERING — PLM</t>
         </is>
       </c>
+      <c r="L80" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="17" t="inlineStr">
@@ -4699,6 +5266,11 @@
           <t>AGENTIC SDLC TRANSFORMATION</t>
         </is>
       </c>
+      <c r="L81" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="17" t="inlineStr">
@@ -4751,6 +5323,11 @@
           <t>AUTONOMOUS INCIDENT REMEDIATION</t>
         </is>
       </c>
+      <c r="L82" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="17" t="inlineStr">
@@ -4803,6 +5380,11 @@
           <t>APPLICATION PERFORMANCE MANAGEMENT</t>
         </is>
       </c>
+      <c r="L83" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="17" t="inlineStr">
@@ -4855,6 +5437,11 @@
           <t>COMMAND CENTER &amp; NETWORK OPERATIONS SECURITY</t>
         </is>
       </c>
+      <c r="L84" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="17" t="inlineStr">
@@ -4907,6 +5494,11 @@
           <t>MULTI-CLOUD GOVERNANCE &amp; INTEGRATION FRAMEWORK</t>
         </is>
       </c>
+      <c r="L85" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="17" t="inlineStr">
@@ -4954,6 +5546,11 @@
           <t>INTELLIGENT ENTERPRISE ORCHESTRATION</t>
         </is>
       </c>
+      <c r="L86" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="17" t="inlineStr">
@@ -5006,6 +5603,11 @@
           <t>AGENTIC AI GOVERNANCE IMPLEMENTATION</t>
         </is>
       </c>
+      <c r="L87" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="17" t="inlineStr">
@@ -5058,6 +5660,11 @@
           <t>LLMOPS AND GENAI OBSERVABILITY</t>
         </is>
       </c>
+      <c r="L88" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="17" t="inlineStr">
@@ -5105,6 +5712,11 @@
           <t>AI GOVERNANCE AND GUARDRAILS</t>
         </is>
       </c>
+      <c r="L89" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="17" t="inlineStr">
@@ -5157,6 +5769,11 @@
           <t>SAM AND HAM — IT ASSET MANAGEMENT</t>
         </is>
       </c>
+      <c r="L90" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" s="17" t="inlineStr">
@@ -5209,6 +5826,11 @@
           <t>DEVSECOPS PIPELINE FOR OPEN BANKING — BFSI</t>
         </is>
       </c>
+      <c r="L91" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="17" t="inlineStr">
@@ -5261,6 +5883,11 @@
           <t>AGENTIC ORDER-TO-CASH TRANSFORMATION</t>
         </is>
       </c>
+      <c r="L92" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="17" t="inlineStr">
@@ -5313,6 +5940,11 @@
           <t>CLOSE AND CONTROL COPILOT</t>
         </is>
       </c>
+      <c r="L93" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" s="17" t="inlineStr">
@@ -5365,6 +5997,11 @@
           <t>AI/ML AND INTELLIGENT AUTOMATION — FINANCIAL INSTITUTIONS</t>
         </is>
       </c>
+      <c r="L94" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="17" t="inlineStr">
@@ -5417,6 +6054,11 @@
           <t>AI-POWERED FINANCIAL RECONCILIATION</t>
         </is>
       </c>
+      <c r="L95" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="17" t="inlineStr">
@@ -5469,6 +6111,11 @@
           <t>MARKET DATA COST OPTIMIZATION &amp; CONVERSATIONAL ANALYTICS</t>
         </is>
       </c>
+      <c r="L96" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="17" t="inlineStr">
@@ -5521,6 +6168,11 @@
           <t>CLEARSIGHT — CHEQUE CLEARING AUTOMATION</t>
         </is>
       </c>
+      <c r="L97" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" s="17" t="inlineStr">
@@ -5573,6 +6225,11 @@
           <t>CONTACTFLOW AI — CONTACT CENTER INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L98" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="17" t="inlineStr">
@@ -5625,6 +6282,11 @@
           <t>VOICEVISTA — CALL INTELLIGENCE &amp; QA AUTOMATION</t>
         </is>
       </c>
+      <c r="L99" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="17" t="inlineStr">
@@ -5672,6 +6334,11 @@
           <t>DUE DILIGENCE ACCELERATION</t>
         </is>
       </c>
+      <c r="L100" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="17" t="inlineStr">
@@ -5724,6 +6391,11 @@
           <t>INVESTMENT ANALYSIS AND MEMO INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L101" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="17" t="inlineStr">
@@ -5771,6 +6443,11 @@
           <t>PORTFOLIO COMPANY MONITORING</t>
         </is>
       </c>
+      <c r="L102" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="17" t="inlineStr">
@@ -5823,6 +6500,11 @@
           <t>COMPLIANCE AND REPORTING AUTOMATION — INVESTMENT FUNDS</t>
         </is>
       </c>
+      <c r="L103" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="17" t="inlineStr">
@@ -5875,6 +6557,11 @@
           <t>DEALIQ — AGENTIC DEAL INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L104" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="17" t="inlineStr">
@@ -5927,6 +6614,11 @@
           <t>OPSIQ — INVESTMENT OPERATIONS CONSOLE</t>
         </is>
       </c>
+      <c r="L105" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="17" t="inlineStr">
@@ -5979,6 +6671,11 @@
           <t>PORTFOLIO INTELLIGENCE AI — CONTINUOUS MONITORING</t>
         </is>
       </c>
+      <c r="L106" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="17" t="inlineStr">
@@ -6031,6 +6728,11 @@
           <t>GENERATION AND GRID FORECASTING INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L107" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="17" t="inlineStr">
@@ -6078,6 +6780,11 @@
           <t>REAL-TIME PROCESS OPTIMIZATION — PETROCHEMICALS</t>
         </is>
       </c>
+      <c r="L108" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="17" t="inlineStr">
@@ -6130,6 +6837,11 @@
           <t>PREDICTIVE ASSET INTELLIGENCE — PROCESS INDUSTRY</t>
         </is>
       </c>
+      <c r="L109" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" s="17" t="inlineStr">
@@ -6182,6 +6894,11 @@
           <t>INDUSTRIAL KNOWLEDGE COPILOT</t>
         </is>
       </c>
+      <c r="L110" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="17" t="inlineStr">
@@ -6234,6 +6951,11 @@
           <t>EDGE AI FOR INDUSTRIAL OPERATIONS</t>
         </is>
       </c>
+      <c r="L111" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="17" t="inlineStr">
@@ -6286,6 +7008,11 @@
           <t>GENERATIVE AI FOR PRODUCT DESIGN</t>
         </is>
       </c>
+      <c r="L112" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="17" t="inlineStr">
@@ -6333,6 +7060,11 @@
           <t>AUTOMATED DMU ANALYSIS AND CHANGE MANAGEMENT</t>
         </is>
       </c>
+      <c r="L113" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="17" t="inlineStr">
@@ -6380,6 +7112,11 @@
           <t>AI-ASSISTED NVH VALIDATION</t>
         </is>
       </c>
+      <c r="L114" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="17" t="inlineStr">
@@ -6432,6 +7169,11 @@
           <t>PLM BUDGET CONTROL AND TESTBED INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L115" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="17" t="inlineStr">
@@ -6484,6 +7226,11 @@
           <t>BOM SYNCHRONIZATION AND VARIANT INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L116" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="17" t="inlineStr">
@@ -6536,6 +7283,11 @@
           <t>ENGINEERING ANALYST AUGMENTATION</t>
         </is>
       </c>
+      <c r="L117" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="17" t="inlineStr">
@@ -6588,6 +7340,11 @@
           <t>PLM COST ESTIMATION &amp; BUDGET GOVERNANCE INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L118" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="17" t="inlineStr">
@@ -6640,6 +7397,11 @@
           <t>WARRANTY &amp; AMC PREDICTIVE COST MODELLING</t>
         </is>
       </c>
+      <c r="L119" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="17" t="inlineStr">
@@ -6692,6 +7454,11 @@
           <t>AI-ASSISTED WARRANTY CLAIM TRIAGE</t>
         </is>
       </c>
+      <c r="L120" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="17" t="inlineStr">
@@ -6744,6 +7511,11 @@
           <t>VISION AI FOR WARRANTY CLAIMS</t>
         </is>
       </c>
+      <c r="L121" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="17" t="inlineStr">
@@ -6796,6 +7568,11 @@
           <t>CONNECTED VEHICLE DATA PLATFORM</t>
         </is>
       </c>
+      <c r="L122" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="17" t="inlineStr">
@@ -6843,6 +7620,11 @@
           <t>TELEMETRY INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L123" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="17" t="inlineStr">
@@ -6895,6 +7677,11 @@
           <t>RANGE PREDICTION AND RANGE POLYGON</t>
         </is>
       </c>
+      <c r="L124" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="17" t="inlineStr">
@@ -6947,6 +7734,11 @@
           <t>BATTERY SOH ANALYTICS AND DEGRADATION INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L125" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="17" t="inlineStr">
@@ -6999,6 +7791,11 @@
           <t>AI-ENABLED DATA EXPLORATION AND REPORTING</t>
         </is>
       </c>
+      <c r="L126" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="17" t="inlineStr">
@@ -7051,6 +7848,11 @@
           <t>INTELLIGENT INVENTORY CONTROL</t>
         </is>
       </c>
+      <c r="L127" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="17" t="inlineStr">
@@ -7103,6 +7905,11 @@
           <t>PREDICTIVE MATERIAL GOVERNANCE</t>
         </is>
       </c>
+      <c r="L128" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="17" t="inlineStr">
@@ -7155,6 +7962,11 @@
           <t>MULTI-JURISDICTIONAL REGULATORY CHANGE INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L129" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="17" t="inlineStr">
@@ -7207,6 +8019,11 @@
           <t>HYBRID TEST AUTOMATION FOR CLINICAL VALIDATION</t>
         </is>
       </c>
+      <c r="L130" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="17" t="inlineStr">
@@ -7259,6 +8076,11 @@
           <t>PLANFORGE AI — AGENTIC PRODUCTION PLANNING</t>
         </is>
       </c>
+      <c r="L131" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="17" t="inlineStr">
@@ -7306,6 +8128,11 @@
           <t>PLANTPULSE — MANUFACTURING OPERATIONS INTELLIGENCE</t>
         </is>
       </c>
+      <c r="L132" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="17" t="inlineStr">
@@ -7358,6 +8185,11 @@
           <t>SERVEIQ — AGENTIC POLICY SERVICING</t>
         </is>
       </c>
+      <c r="L133" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="17" t="inlineStr">
@@ -7410,6 +8242,11 @@
           <t>Transforming Aviation MRO with Predictive Maintenance and AIOps</t>
         </is>
       </c>
+      <c r="L134" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="17" t="inlineStr">
@@ -7462,6 +8299,11 @@
           <t>AI-Pod Engagement Case Study: Northwind Aerospace</t>
         </is>
       </c>
+      <c r="L135" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="17" t="inlineStr">
@@ -7514,56 +8356,859 @@
           <t>AI POD FOR RENEWABLE ENERGY OPTIMIZATION</t>
         </is>
       </c>
+      <c r="L136" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
     </row>
     <row r="137">
-      <c r="A137" t="inlineStr">
+      <c r="A137" s="17" t="inlineStr">
         <is>
           <t>CS136</t>
         </is>
       </c>
-      <c r="B137" t="inlineStr">
+      <c r="B137" s="17" t="inlineStr">
         <is>
           <t>WORKFORCE</t>
         </is>
       </c>
-      <c r="C137" t="inlineStr">
-        <is>
-          <t>CASE_STUDY</t>
-        </is>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>IF industry/function/keywords match context or transcript</t>
-        </is>
-      </c>
-      <c r="F137" t="inlineStr">
+      <c r="C137" s="17" t="inlineStr">
+        <is>
+          <t>CASE_STUDY</t>
+        </is>
+      </c>
+      <c r="E137" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
+      <c r="F137" s="17" t="inlineStr">
         <is>
           <t>WORKFORCE</t>
         </is>
       </c>
-      <c r="G137" t="inlineStr">
+      <c r="G137" s="17" t="inlineStr">
         <is>
           <t>ENERGY</t>
         </is>
       </c>
-      <c r="H137" t="inlineStr">
+      <c r="H137" s="17" t="inlineStr">
         <is>
           <t>DATA_AI_PLATFORM</t>
         </is>
       </c>
-      <c r="I137" t="inlineStr">
+      <c r="I137" s="17" t="inlineStr">
         <is>
           <t>Energy · Grid Operations · AI Pod · Renewable Dispatch · Curtailment Reduction · Data Engineering</t>
         </is>
       </c>
-      <c r="J137" t="inlineStr">
-        <is>
-          <t>AUTO</t>
-        </is>
-      </c>
-      <c r="K137" t="inlineStr">
+      <c r="J137" s="17" t="inlineStr">
+        <is>
+          <t>AUTO</t>
+        </is>
+      </c>
+      <c r="K137" s="17" t="inlineStr">
         <is>
           <t>AI-DRIVEN GRID OPTIMIZATION FOR RENEWABLES</t>
+        </is>
+      </c>
+      <c r="L137" s="17" t="inlineStr">
+        <is>
+          <t>IF industry/function/keywords match context or transcript</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" s="17" t="inlineStr">
+        <is>
+          <t>CS02B</t>
+        </is>
+      </c>
+      <c r="B138" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C138" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D138" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="E138" s="17" t="inlineStr">
+        <is>
+          <t>SPECIAL - see matcher._SPECIAL_STAGE_RULES</t>
+        </is>
+      </c>
+      <c r="F138" s="17" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="J138" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K138" s="17" t="inlineStr">
+        <is>
+          <t>WHO WE ARE</t>
+        </is>
+      </c>
+      <c r="L138" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=Y--, wt=MS, trigger=none)</t>
+        </is>
+      </c>
+      <c r="M138" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="P138" s="17" t="inlineStr">
+        <is>
+          <t>pure</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" s="17" t="inlineStr">
+        <is>
+          <t>CS137</t>
+        </is>
+      </c>
+      <c r="B139" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C139" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D139" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="E139" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="J139" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K139" s="17" t="inlineStr">
+        <is>
+          <t>GLOBAL FOOTPRINT &amp; INDUSTRIES WE SERVE</t>
+        </is>
+      </c>
+      <c r="L139" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="M139" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N139" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O139" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q139" s="17" t="inlineStr">
+        <is>
+          <t>gcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" s="17" t="inlineStr">
+        <is>
+          <t>CS138</t>
+        </is>
+      </c>
+      <c r="B140" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C140" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D140" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="E140" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="J140" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K140" s="17" t="inlineStr">
+        <is>
+          <t>END TO END GCC BUILD OFFERINGS</t>
+        </is>
+      </c>
+      <c r="L140" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="M140" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N140" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O140" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q140" s="17" t="inlineStr">
+        <is>
+          <t>gcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" s="17" t="inlineStr">
+        <is>
+          <t>CS139</t>
+        </is>
+      </c>
+      <c r="B141" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="C141" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D141" s="17" t="inlineStr">
+        <is>
+          <t>CORE</t>
+        </is>
+      </c>
+      <c r="E141" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="J141" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K141" s="17" t="inlineStr">
+        <is>
+          <t>GREENFIELD &amp; BROWNFIELD USE CASES</t>
+        </is>
+      </c>
+      <c r="L141" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=YYY, wt=None, trigger=gcc)</t>
+        </is>
+      </c>
+      <c r="M141" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="N141" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O141" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q141" s="17" t="inlineStr">
+        <is>
+          <t>gcc</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" s="17" t="inlineStr">
+        <is>
+          <t>CS140</t>
+        </is>
+      </c>
+      <c r="B142" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C142" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D142" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="E142" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="F142" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J142" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K142" s="17" t="inlineStr">
+        <is>
+          <t>OUR ENGAGEMENT MODEL</t>
+        </is>
+      </c>
+      <c r="L142" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="N142" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O142" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q142" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" s="17" t="inlineStr">
+        <is>
+          <t>CS141</t>
+        </is>
+      </c>
+      <c r="B143" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C143" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D143" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="E143" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="F143" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J143" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K143" s="17" t="inlineStr">
+        <is>
+          <t>CONTRACT PROCESS OUTSOURCING OPERATING MODEL</t>
+        </is>
+      </c>
+      <c r="L143" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="N143" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O143" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q143" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" s="17" t="inlineStr">
+        <is>
+          <t>CS142</t>
+        </is>
+      </c>
+      <c r="B144" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C144" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D144" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="E144" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="F144" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J144" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K144" s="17" t="inlineStr">
+        <is>
+          <t>39</t>
+        </is>
+      </c>
+      <c r="L144" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=WORKFORCE, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="N144" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O144" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q144" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" s="17" t="inlineStr">
+        <is>
+          <t>CS143</t>
+        </is>
+      </c>
+      <c r="B145" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C145" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D145" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E145" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="F145" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J145" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K145" s="17" t="inlineStr">
+        <is>
+          <t>LIFECYCLE FOR OPERATIONS</t>
+        </is>
+      </c>
+      <c r="L145" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="Q145" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" s="17" t="inlineStr">
+        <is>
+          <t>CS144</t>
+        </is>
+      </c>
+      <c r="B146" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C146" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D146" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E146" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="F146" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J146" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K146" s="17" t="inlineStr">
+        <is>
+          <t>ENGAGEMENT &amp; RETENTION OPERATING MODEL</t>
+        </is>
+      </c>
+      <c r="L146" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="Q146" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" s="17" t="inlineStr">
+        <is>
+          <t>CS145</t>
+        </is>
+      </c>
+      <c r="B147" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="C147" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D147" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E147" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="F147" s="17" t="inlineStr">
+        <is>
+          <t>WORKFORCE</t>
+        </is>
+      </c>
+      <c r="J147" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K147" s="17" t="inlineStr">
+        <is>
+          <t>COMPETITIVE ADVANTAGES AT SCALE – EXECUTION PROOF POINTS</t>
+        </is>
+      </c>
+      <c r="L147" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=WORKFORCE, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="Q147" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" s="17" t="inlineStr">
+        <is>
+          <t>CS146</t>
+        </is>
+      </c>
+      <c r="B148" s="17" t="inlineStr">
+        <is>
+          <t>AI_POD</t>
+        </is>
+      </c>
+      <c r="C148" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D148" s="17" t="inlineStr">
+        <is>
+          <t>AI_POD</t>
+        </is>
+      </c>
+      <c r="E148" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=AI_POD, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="F148" s="17" t="inlineStr">
+        <is>
+          <t>AI_POD</t>
+        </is>
+      </c>
+      <c r="J148" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K148" s="17" t="inlineStr">
+        <is>
+          <t>AI PODS + INTERVIEW-AS-A-SERVICE</t>
+        </is>
+      </c>
+      <c r="L148" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=AI_POD, trigger=asked)</t>
+        </is>
+      </c>
+      <c r="N148" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O148" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="Q148" s="17" t="inlineStr">
+        <is>
+          <t>asked</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" s="17" t="inlineStr">
+        <is>
+          <t>CS147</t>
+        </is>
+      </c>
+      <c r="B149" s="17" t="inlineStr">
+        <is>
+          <t>CASE_STUDIES</t>
+        </is>
+      </c>
+      <c r="C149" s="17" t="inlineStr">
+        <is>
+          <t>DIVIDER</t>
+        </is>
+      </c>
+      <c r="D149" s="17" t="inlineStr">
+        <is>
+          <t>CASE_STUDIES</t>
+        </is>
+      </c>
+      <c r="E149" s="17" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+      <c r="J149" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K149" s="17" t="inlineStr">
+        <is>
+          <t>CASE STUDIES</t>
+        </is>
+      </c>
+      <c r="L149" t="inlineStr">
+        <is>
+          <t>ALWAYS</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" s="17" t="inlineStr">
+        <is>
+          <t>CS148</t>
+        </is>
+      </c>
+      <c r="B150" s="17" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="C150" s="17" t="inlineStr">
+        <is>
+          <t>STANDARD</t>
+        </is>
+      </c>
+      <c r="D150" s="17" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="E150" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=MS, trigger=none)</t>
+        </is>
+      </c>
+      <c r="F150" s="17" t="inlineStr">
+        <is>
+          <t>MS</t>
+        </is>
+      </c>
+      <c r="J150" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K150" s="17" t="inlineStr">
+        <is>
+          <t>How We Move Forward</t>
+        </is>
+      </c>
+      <c r="L150" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=-YY, wt=MS, trigger=none)</t>
+        </is>
+      </c>
+      <c r="N150" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+      <c r="O150" s="17" t="inlineStr">
+        <is>
+          <t>Y</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" s="17" t="inlineStr">
+        <is>
+          <t>CS149</t>
+        </is>
+      </c>
+      <c r="B151" s="17" t="inlineStr">
+        <is>
+          <t>APPENDIX</t>
+        </is>
+      </c>
+      <c r="C151" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="D151" s="17" t="inlineStr">
+        <is>
+          <t>OPTIONAL</t>
+        </is>
+      </c>
+      <c r="E151" s="17" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=None, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="J151" s="17" t="inlineStr">
+        <is>
+          <t>MANUAL</t>
+        </is>
+      </c>
+      <c r="K151" s="17" t="inlineStr">
+        <is>
+          <t>APPENDIX</t>
+        </is>
+      </c>
+      <c r="L151" t="inlineStr">
+        <is>
+          <t>STAGE_RULE (stage=---, wt=None, trigger=manual)</t>
+        </is>
+      </c>
+      <c r="Q151" s="17" t="inlineStr">
+        <is>
+          <t>manual</t>
         </is>
       </c>
     </row>

</xml_diff>